<commit_message>
new howell file naming
</commit_message>
<xml_diff>
--- a/mitchell10x3.xlsx
+++ b/mitchell10x3.xlsx
@@ -499,7 +499,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>For public domain. No rights reserved. Generated on Apr 23, 2026.</t>
+          <t>For public domain. No rights reserved. Generated on Jun 18, 2026.</t>
         </is>
       </c>
     </row>
@@ -573,12 +573,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Name 24</t>
+          <t>Name 90</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Name 84</t>
+          <t>Name 22</t>
         </is>
       </c>
       <c r="D9" s="4">
@@ -596,12 +596,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Name 56</t>
+          <t>Name 86</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Name 42</t>
+          <t>Name 15</t>
         </is>
       </c>
       <c r="D10" s="4">
@@ -619,12 +619,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Name 57</t>
+          <t>Name 63</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Name 21</t>
+          <t>Name 47</t>
         </is>
       </c>
       <c r="D11" s="4">
@@ -642,12 +642,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Name 58</t>
+          <t>Name 14</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Name 82</t>
+          <t>Name 90</t>
         </is>
       </c>
       <c r="D12" s="4">
@@ -665,12 +665,12 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Name 70</t>
+          <t>Name 13</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Name 34</t>
+          <t>Name 28</t>
         </is>
       </c>
       <c r="D13" s="8">
@@ -721,12 +721,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Name 19</t>
+          <t>Name 80</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Name 22</t>
+          <t>Name 66</t>
         </is>
       </c>
       <c r="D17" s="4">
@@ -744,12 +744,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Name 58</t>
+          <t>Name 72</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Name 47</t>
+          <t>Name 76</t>
         </is>
       </c>
       <c r="D18" s="4">
@@ -767,12 +767,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Name 89</t>
+          <t>Name 38</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Name 46</t>
+          <t>Name 82</t>
         </is>
       </c>
       <c r="D19" s="4">
@@ -790,12 +790,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Name 81</t>
+          <t>Name 34</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Name 22</t>
+          <t>Name 21</t>
         </is>
       </c>
       <c r="D20" s="4">
@@ -813,12 +813,12 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Name 73</t>
+          <t>Name 26</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Name 46</t>
+          <t>Name 48</t>
         </is>
       </c>
       <c r="D21" s="8">

</xml_diff>